<commit_message>
data: update 고객사계측기현황.xlsx for 2026-08-28
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/고객사계측기현황.xlsx
+++ b/docs/dashboard/data/고객사계측기현황.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K47"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -174,17 +174,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>(주)대성티엠씨</t>
+          <t>디지트론</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>경기도 성남시 수정구</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>6068641818</t>
+          <t>1298603001</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -197,7 +197,7 @@
         <v>0.0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>19.0</v>
+        <v>144.0</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0.0</v>
@@ -217,30 +217,30 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>오씨아이파워주식회사</t>
+          <t>현대건설(주)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>전북특별자치도 군산시</t>
+          <t>경상북도 울진군</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>1048644532</t>
+          <t>1018116293</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>53.0</v>
+        <v>5.0</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0.0</v>
@@ -260,17 +260,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>세일전장 주식회사</t>
+          <t>(주)대성티엠씨</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>충청남도 홍성군</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2218802452</t>
+          <t>6068641818</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
@@ -283,7 +283,7 @@
         <v>0.0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>190.0</v>
+        <v>19.0</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0.0</v>
@@ -303,17 +303,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>(주)동광보일러</t>
+          <t>오씨아이파워주식회사</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>전북특별자치도 군산시</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1408121883</t>
+          <t>1048644532</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
@@ -326,7 +326,7 @@
         <v>0.0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>37.0</v>
+        <v>53.0</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0.0</v>
@@ -346,17 +346,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>(주)센추리 아산공장</t>
+          <t>세일전장 주식회사</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>충청남도 홍성군</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>3128545076</t>
+          <t>2218802452</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -369,7 +369,7 @@
         <v>0.0</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>179.0</v>
+        <v>190.0</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>0.0</v>
@@ -389,7 +389,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에이치엔에프</t>
+          <t>(주)동광보일러</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -399,7 +399,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>7398801954</t>
+          <t>1408121883</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -412,7 +412,7 @@
         <v>0.0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>223.0</v>
+        <v>37.0</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>0.0</v>
@@ -432,17 +432,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
+          <t>(주)센추리 아산공장</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>8858800321</t>
+          <t>3128545076</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -455,7 +455,7 @@
         <v>0.0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>23.0</v>
+        <v>179.0</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>0.0</v>
@@ -475,17 +475,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
+          <t>주식회사 에이치엔에프</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 동탄구</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>7888101296</t>
+          <t>7398801954</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -498,7 +498,7 @@
         <v>0.0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>121.0</v>
+        <v>223.0</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>0.0</v>
@@ -518,17 +518,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
+          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 동대문구</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>5318701197</t>
+          <t>8858800321</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
@@ -541,7 +541,7 @@
         <v>0.0</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>118.0</v>
+        <v>23.0</v>
       </c>
       <c r="H10" s="2" t="n">
         <v>0.0</v>
@@ -561,17 +561,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>태광푸드(주)</t>
+          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>경기도 파주시</t>
+          <t>경기도 화성시 동탄구</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>1508701192</t>
+          <t>7888101296</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
@@ -584,7 +584,7 @@
         <v>0.0</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>49.0</v>
+        <v>121.0</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>0.0</v>
@@ -604,17 +604,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>노을그린에너지 주식회사</t>
+          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 마포구</t>
+          <t>서울특별시 동대문구</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>1058807174</t>
+          <t>5318701197</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
@@ -627,7 +627,7 @@
         <v>0.0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>19.0</v>
+        <v>118.0</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>0.0</v>
@@ -647,17 +647,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>김포골드라인에스알에스 주식회사</t>
+          <t>태광푸드(주)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>경기도 파주시</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>6258803309</t>
+          <t>1508701192</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
@@ -670,7 +670,7 @@
         <v>0.0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>58.0</v>
+        <v>49.0</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>0.0</v>
@@ -690,17 +690,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>주식회사 싱크홀</t>
+          <t>노을그린에너지 주식회사</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울특별시 마포구</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>6798502456</t>
+          <t>1058807174</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
@@ -713,7 +713,7 @@
         <v>0.0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>9.0</v>
+        <v>19.0</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>0.0</v>
@@ -733,17 +733,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>대동도어주식회사</t>
+          <t>김포골드라인에스알에스 주식회사</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>1348173163</t>
+          <t>6258803309</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
@@ -756,7 +756,7 @@
         <v>0.0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>191.0</v>
+        <v>58.0</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>0.0</v>
@@ -776,17 +776,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>지티엑스에이운영(주)</t>
+          <t>주식회사 싱크홀</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>경기도 고양시 덕양구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>8738702917</t>
+          <t>6798502456</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -799,7 +799,7 @@
         <v>0.0</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>12.0</v>
+        <v>9.0</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>0.0</v>
@@ -819,17 +819,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>영상폴리텍</t>
+          <t>대동도어주식회사</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>인천광역시 연수구</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>1312660786</t>
+          <t>1348173163</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
@@ -842,7 +842,7 @@
         <v>0.0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>70.0</v>
+        <v>165.0</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>0.0</v>
@@ -862,17 +862,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>주식회사 파라타항공</t>
+          <t>지티엑스에이운영(주)</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>강원특별자치도 양양군</t>
+          <t>경기도 고양시 덕양구</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>7108100367</t>
+          <t>8738702917</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
@@ -885,7 +885,7 @@
         <v>0.0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>71.0</v>
+        <v>12.0</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>0.0</v>
@@ -905,17 +905,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>대한약품공업(주)반월공장</t>
+          <t>영상폴리텍</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>1348500111</t>
+          <t>1312660786</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
@@ -928,7 +928,7 @@
         <v>0.0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>82.0</v>
+        <v>70.0</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>0.0</v>
@@ -948,17 +948,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>주식회사 대솔오시스</t>
+          <t>대한약품공업(주)반월공장</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>1398115533</t>
+          <t>1348500111</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
@@ -971,7 +971,7 @@
         <v>0.0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>37.0</v>
+        <v>82.0</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>0.0</v>
@@ -991,17 +991,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>케이젯정밀 (주) 펌프공장</t>
+          <t>주식회사 대솔오시스</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>1348501217</t>
+          <t>1398115533</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
@@ -1014,7 +1014,7 @@
         <v>0.0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>208.0</v>
+        <v>37.0</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>0.0</v>
@@ -1034,17 +1034,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>케이젯정밀 (주) 밸브공장</t>
+          <t>(주) 대한솔루션</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>1348555479</t>
+          <t>1398100699</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
@@ -1057,7 +1057,7 @@
         <v>0.0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>157.0</v>
+        <v>47.0</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>0.0</v>
@@ -1077,7 +1077,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>(주) 대한솔루션</t>
+          <t>(주)오성기전</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>1398100699</t>
+          <t>1318629038</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
@@ -1100,7 +1100,7 @@
         <v>0.0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>47.0</v>
+        <v>44.0</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>0.0</v>
@@ -1120,30 +1120,30 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>(주)오성기전</t>
+          <t>(주)윤성에프앤씨</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안성시</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>1318629038</t>
+          <t>1348150350</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>0.0</v>
+        <v>288.0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0</v>
+        <v>288.0</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>44.0</v>
+        <v>214.0</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>0.0</v>
@@ -1152,7 +1152,7 @@
         <v>0.0</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>0.0</v>
+        <v>73.0</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -1163,30 +1163,30 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>(주)윤성에프앤씨</t>
+          <t>(주)백콤</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>경기도 안성시</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>1348150350</t>
+          <t>1308628716</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>0.0</v>
+        <v>47.0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.0</v>
+        <v>47.0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>214.0</v>
+        <v>27.0</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>0.0</v>
@@ -1206,39 +1206,39 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>(주)백콤</t>
+          <t>한국미쓰비시엘리베이터(주)</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>인천광역시 연수구</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>1308628716</t>
+          <t>1378514007</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>47.0</v>
+        <v>209.0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>47.0</v>
+        <v>209.0</v>
       </c>
       <c r="F26" s="2" t="n">
+        <v>92.0</v>
+      </c>
+      <c r="G26" s="2" t="n">
+        <v>128.0</v>
+      </c>
+      <c r="H26" s="2" t="n">
         <v>10.0</v>
       </c>
-      <c r="G26" s="2" t="n">
-        <v>27.0</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I26" s="2" t="n">
-        <v>0.0</v>
+        <v>17.0</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -1249,39 +1249,39 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>한국미쓰비시엘리베이터(주)</t>
+          <t>비카코리아 주식회사</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>1378514007</t>
+          <t>6108128707</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>209.0</v>
+        <v>0.0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>209.0</v>
+        <v>0.0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>92.0</v>
+        <v>0.0</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>128.0</v>
+        <v>107.0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>17.0</v>
+        <v>0.0</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
@@ -1292,39 +1292,39 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>비카코리아 주식회사</t>
+          <t>(주)디바이스</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>충청남도 천안시 서북구</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>6108128707</t>
+          <t>3128157991</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="F28" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>107.0</v>
+        <v>70.0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>0.0</v>
+        <v>17.0</v>
       </c>
       <c r="I28" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>0.0</v>
+        <v>51.0</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -1335,39 +1335,39 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>(주)디바이스</t>
+          <t>(주)지에프에스</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>충청남도 천안시 서북구</t>
+          <t>경기도 의정부시</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>3128157991</t>
+          <t>1278107419</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>70.0</v>
+        <v>0.0</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>70.0</v>
+        <v>0.0</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>70.0</v>
+        <v>104.0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>16.0</v>
+        <v>0.0</v>
       </c>
       <c r="I29" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>51.0</v>
+        <v>0.0</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -1378,39 +1378,39 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>(주)지에프에스</t>
+          <t>(주)케이피씨엠</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>경기도 의정부시</t>
+          <t>경상북도 경산시</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>1278107419</t>
+          <t>5158140973</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>0.0</v>
+        <v>188.0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0</v>
+        <v>188.0</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>104.0</v>
+        <v>174.0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>0.0</v>
+        <v>25.0</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
@@ -1421,39 +1421,39 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>(주)케이피씨엠</t>
+          <t>(주)경인기술</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>경상북도 경산시</t>
+          <t>서울특별시 영등포구</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>5158140973</t>
+          <t>1138156416</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>188.0</v>
+        <v>0.0</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>188.0</v>
+        <v>0.0</v>
       </c>
       <c r="F31" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>174.0</v>
+        <v>35.0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>27.0</v>
+        <v>0.0</v>
       </c>
       <c r="J31" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
@@ -1464,17 +1464,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>(주)경인기술</t>
+          <t>(주)코리아하이텍</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 영등포구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>1138156416</t>
+          <t>1348106311</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
@@ -1487,7 +1487,7 @@
         <v>0.0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>35.0</v>
+        <v>296.0</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>0.0</v>
@@ -1507,30 +1507,30 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>(주)코리아하이텍</t>
+          <t>에브제트아시아(주)</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>서울특별시 강서구</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>1348106311</t>
+          <t>1208731282</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>296.0</v>
+        <v>70.0</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>0.0</v>
@@ -1550,39 +1550,39 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>에브제트아시아(주)</t>
+          <t>디엔엠항공</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 강서구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>1208731282</t>
+          <t>6131783159</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>1.0</v>
+        <v>452.0</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>1.0</v>
+        <v>315.0</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>70.0</v>
+        <v>243.0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>0.0</v>
+        <v>22.0</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>0.0</v>
+        <v>44.0</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -1593,39 +1593,39 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>디엔엠항공</t>
+          <t>씨트론(주)</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>인천광역시 계양구</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>6131783159</t>
+          <t>1228159023</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>452.0</v>
+        <v>0.0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>315.0</v>
+        <v>0.0</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>243.0</v>
+        <v>41.0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>22.0</v>
+        <v>0.0</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>44.0</v>
+        <v>0.0</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
@@ -1636,17 +1636,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>씨트론(주)</t>
+          <t>(주)알피바이오</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 계양구</t>
+          <t>경기도 화성시 만세구</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>1228159023</t>
+          <t>7758501361</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
@@ -1659,7 +1659,7 @@
         <v>0.0</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>41.0</v>
+        <v>10.0</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>0.0</v>
@@ -1679,30 +1679,30 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>(주)알피바이오</t>
+          <t>주식회사 코젠바이오텍</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 만세구</t>
+          <t>서울특별시 금천구</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>7758501361</t>
+          <t>1018156320</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>0.0</v>
+        <v>45.0</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.0</v>
+        <v>45.0</v>
       </c>
       <c r="F37" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>10.0</v>
+        <v>150.0</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>0.0</v>
@@ -1722,39 +1722,39 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>주식회사 코젠바이오텍</t>
+          <t>(주)에어로피스</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 금천구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>1018156320</t>
+          <t>1378604165</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>45.0</v>
+        <v>237.0</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>45.0</v>
+        <v>237.0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>0.0</v>
+        <v>57.0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>150.0</v>
+        <v>176.0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>0.0</v>
+        <v>30.0</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>0.0</v>
+        <v>27.0</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>0.0</v>
+        <v>86.0</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -1765,39 +1765,39 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>(주)에어로피스</t>
+          <t>주식회사 덱스레보</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울 금천구</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>1378604165</t>
+          <t>1198678150</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>237.0</v>
+        <v>10.0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>237.0</v>
+        <v>10.0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>57.0</v>
+        <v>0.0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>176.0</v>
+        <v>160.0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>29.0</v>
+        <v>0.0</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>27.0</v>
+        <v>0.0</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>86.0</v>
+        <v>0.0</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
@@ -1808,36 +1808,36 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>주식회사 덱스레보</t>
+          <t>주식회사 카프마이크로</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>서울 금천구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>1198678150</t>
+          <t>3148613655</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>10.0</v>
+        <v>60.0</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>10.0</v>
+        <v>60.0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>0.0</v>
+        <v>17.0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>160.0</v>
+        <v>33.0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>0.0</v>
+        <v>14.0</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.0</v>
@@ -1851,39 +1851,39 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>주식회사 카프마이크로</t>
+          <t>연합정밀(주)</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>충남 천안시 동남구</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>3148613655</t>
+          <t>3128109219</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>60.0</v>
+        <v>1827.0</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>60.0</v>
+        <v>1827.0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>17.0</v>
+        <v>525.0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>33.0</v>
+        <v>7.0</v>
       </c>
       <c r="H41" s="2" t="n">
         <v>1.0</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>14.0</v>
+        <v>0.0</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>0.0</v>
+        <v>18.0</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -1894,39 +1894,39 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>연합정밀(주)</t>
+          <t>(주)우리기술</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>충남 천안시 동남구</t>
+          <t>서울 마포구</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>3128109219</t>
+          <t>1128138619</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>1827.0</v>
+        <v>84.0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>1827.0</v>
+        <v>84.0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>525.0</v>
+        <v>22.0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>7.0</v>
+        <v>71.0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I42" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>18.0</v>
+        <v>0.0</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -1937,33 +1937,33 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>(주)우리기술</t>
+          <t>(주)신화프리텍</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>서울 마포구</t>
+          <t>경남 창원시 성산구</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>1128138619</t>
+          <t>6088151660</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>84.0</v>
+        <v>1070.0</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>84.0</v>
+        <v>1051.0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>22.0</v>
+        <v>111.0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>71.0</v>
+        <v>1523.0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>0.0</v>
+        <v>39.0</v>
       </c>
       <c r="I43" s="2" t="n">
         <v>0.0</v>
@@ -1980,39 +1980,39 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>(주)신화프리텍</t>
+          <t>(주)한국기능공사</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>경남 창원시 성산구</t>
+          <t>충북 음성군</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>6088151660</t>
+          <t>1258112293</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>1070.0</v>
+        <v>614.0</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>1051.0</v>
+        <v>614.0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>111.0</v>
+        <v>250.0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>1525.0</v>
+        <v>309.0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>39.0</v>
+        <v>3.0</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0.0</v>
+        <v>8.0</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>0.0</v>
+        <v>376.0</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -2023,39 +2023,39 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>(주)한국기능공사</t>
+          <t>(주)휴니드테크놀러지스</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>충북 음성군</t>
+          <t>인천 연수구</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>1258112293</t>
+          <t>1238106174</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>614.0</v>
+        <v>916.0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>614.0</v>
+        <v>916.0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>250.0</v>
+        <v>128.0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>309.0</v>
+        <v>871.0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>3.0</v>
+        <v>40.0</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>8.0</v>
+        <v>42.0</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>376.0</v>
+        <v>145.0</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -2066,84 +2066,41 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>(주)휴니드테크놀러지스</t>
+          <t>(주)서연이화 아산공장</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>인천 연수구</t>
+          <t>충남 아산시</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>1238106174</t>
+          <t>3128564374</t>
         </is>
       </c>
       <c r="D46" s="2" t="n">
-        <v>916.0</v>
+        <v>84.0</v>
       </c>
       <c r="E46" s="2" t="n">
-        <v>916.0</v>
+        <v>84.0</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>128.0</v>
+        <v>5.0</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>871.0</v>
+        <v>47.0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>40.0</v>
+        <v>0.0</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>42.0</v>
+        <v>0.0</v>
       </c>
       <c r="J46" s="2" t="n">
-        <v>145.0</v>
+        <v>0.0</v>
       </c>
       <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>(주)서연이화 아산공장</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>충남 아산시</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>3128564374</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="n">
-        <v>84.0</v>
-      </c>
-      <c r="E47" s="2" t="n">
-        <v>84.0</v>
-      </c>
-      <c r="F47" s="2" t="n">
-        <v>5.0</v>
-      </c>
-      <c r="G47" s="2" t="n">
-        <v>48.0</v>
-      </c>
-      <c r="H47" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="I47" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J47" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>

<commit_message>
data: update 고객사계측기현황.xlsx for 2026-09-04
</commit_message>
<xml_diff>
--- a/docs/dashboard/data/고객사계측기현황.xlsx
+++ b/docs/dashboard/data/고객사계측기현황.xlsx
@@ -98,7 +98,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K46"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -174,30 +174,30 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>디지트론</t>
+          <t>하이에어코리아(주)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>경기도 성남시 수정구</t>
+          <t>경상남도 김해시</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>1298603001</t>
+          <t>6038110081</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.0</v>
+        <v>11.0</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.0</v>
+        <v>11.0</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>144.0</v>
+        <v>438.0</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>0.0</v>
@@ -217,30 +217,30 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>현대건설(주)</t>
+          <t>보그워너충주 유한책임회사</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>경상북도 울진군</t>
+          <t>충청북도 충주시</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>1018116293</t>
+          <t>3038108176</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5.0</v>
+        <v>284.0</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>0.0</v>
@@ -260,30 +260,30 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>(주)대성티엠씨</t>
+          <t>디지트론</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>경기도 성남시 수정구</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>6068641818</t>
+          <t>1298603001</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.0</v>
+        <v>10.0</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>19.0</v>
+        <v>182.0</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0.0</v>
@@ -303,30 +303,30 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>오씨아이파워주식회사</t>
+          <t>현대건설(주)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>전북특별자치도 군산시</t>
+          <t>경상북도 울진군</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>1048644532</t>
+          <t>1018116293</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>53.0</v>
+        <v>30.0</v>
       </c>
       <c r="H5" s="2" t="n">
         <v>0.0</v>
@@ -346,17 +346,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>세일전장 주식회사</t>
+          <t>(주)대성티엠씨</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>충청남도 홍성군</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2218802452</t>
+          <t>6068641818</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -369,7 +369,7 @@
         <v>0.0</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>190.0</v>
+        <v>19.0</v>
       </c>
       <c r="H6" s="2" t="n">
         <v>0.0</v>
@@ -389,17 +389,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>(주)동광보일러</t>
+          <t>오씨아이파워주식회사</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>전북특별자치도 군산시</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>1408121883</t>
+          <t>1048644532</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
@@ -412,7 +412,7 @@
         <v>0.0</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>37.0</v>
+        <v>53.0</v>
       </c>
       <c r="H7" s="2" t="n">
         <v>0.0</v>
@@ -432,17 +432,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>(주)센추리 아산공장</t>
+          <t>세일전장 주식회사</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>충청남도 아산시</t>
+          <t>충청남도 홍성군</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>3128545076</t>
+          <t>2218802452</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
@@ -455,7 +455,7 @@
         <v>0.0</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>179.0</v>
+        <v>190.0</v>
       </c>
       <c r="H8" s="2" t="n">
         <v>0.0</v>
@@ -475,7 +475,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에이치엔에프</t>
+          <t>(주)동광보일러</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -485,7 +485,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>7398801954</t>
+          <t>1408121883</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
@@ -498,7 +498,7 @@
         <v>0.0</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>223.0</v>
+        <v>37.0</v>
       </c>
       <c r="H9" s="2" t="n">
         <v>0.0</v>
@@ -518,39 +518,39 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
+          <t>(주)센추리 아산공장</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>8858800321</t>
+          <t>3128545076</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0.0</v>
+        <v>293.0</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.0</v>
+        <v>293.0</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>0.0</v>
+        <v>54.0</v>
       </c>
       <c r="G10" s="2" t="n">
+        <v>179.0</v>
+      </c>
+      <c r="H10" s="2" t="n">
         <v>23.0</v>
       </c>
-      <c r="H10" s="2" t="n">
-        <v>0.0</v>
-      </c>
       <c r="I10" s="2" t="n">
-        <v>0.0</v>
+        <v>21.0</v>
       </c>
       <c r="J10" s="2" t="n">
-        <v>0.0</v>
+        <v>226.0</v>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
@@ -561,17 +561,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
+          <t>주식회사 에이치엔에프</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 동탄구</t>
+          <t>충청남도 아산시</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>7888101296</t>
+          <t>7398801954</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
@@ -584,7 +584,7 @@
         <v>0.0</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>121.0</v>
+        <v>223.0</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>0.0</v>
@@ -604,17 +604,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
+          <t>주식회사 브이티이코리아(VTE KOREA Co., Ltd)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 동대문구</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>5318701197</t>
+          <t>8858800321</t>
         </is>
       </c>
       <c r="D12" s="2" t="n">
@@ -627,7 +627,7 @@
         <v>0.0</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>118.0</v>
+        <v>23.0</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>0.0</v>
@@ -647,17 +647,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>태광푸드(주)</t>
+          <t>주식회사 에스지에스코리아(SGS KOREA CO.,LTD.)</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>경기도 파주시</t>
+          <t>경기도 화성시 동탄구</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>1508701192</t>
+          <t>7888101296</t>
         </is>
       </c>
       <c r="D13" s="2" t="n">
@@ -670,7 +670,7 @@
         <v>0.0</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>49.0</v>
+        <v>81.0</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>0.0</v>
@@ -690,17 +690,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>노을그린에너지 주식회사</t>
+          <t>주식회사 엑소퍼트(EXoPERT CORPORATION)</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 마포구</t>
+          <t>서울특별시 동대문구</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>1058807174</t>
+          <t>5318701197</t>
         </is>
       </c>
       <c r="D14" s="2" t="n">
@@ -713,7 +713,7 @@
         <v>0.0</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>19.0</v>
+        <v>118.0</v>
       </c>
       <c r="H14" s="2" t="n">
         <v>0.0</v>
@@ -733,17 +733,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>김포골드라인에스알에스 주식회사</t>
+          <t>태광푸드(주)</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>경기도 파주시</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>6258803309</t>
+          <t>1508701192</t>
         </is>
       </c>
       <c r="D15" s="2" t="n">
@@ -756,7 +756,7 @@
         <v>0.0</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>58.0</v>
+        <v>49.0</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>0.0</v>
@@ -776,17 +776,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>주식회사 싱크홀</t>
+          <t>노을그린에너지 주식회사</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울특별시 마포구</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>6798502456</t>
+          <t>1058807174</t>
         </is>
       </c>
       <c r="D16" s="2" t="n">
@@ -799,7 +799,7 @@
         <v>0.0</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>9.0</v>
+        <v>19.0</v>
       </c>
       <c r="H16" s="2" t="n">
         <v>0.0</v>
@@ -819,17 +819,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>대동도어주식회사</t>
+          <t>김포골드라인에스알에스 주식회사</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>1348173163</t>
+          <t>6258803309</t>
         </is>
       </c>
       <c r="D17" s="2" t="n">
@@ -842,7 +842,7 @@
         <v>0.0</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>165.0</v>
+        <v>58.0</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>0.0</v>
@@ -862,17 +862,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>지티엑스에이운영(주)</t>
+          <t>주식회사 싱크홀</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>경기도 고양시 덕양구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>8738702917</t>
+          <t>6798502456</t>
         </is>
       </c>
       <c r="D18" s="2" t="n">
@@ -885,7 +885,7 @@
         <v>0.0</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>12.0</v>
+        <v>9.0</v>
       </c>
       <c r="H18" s="2" t="n">
         <v>0.0</v>
@@ -905,17 +905,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>영상폴리텍</t>
+          <t>지티엑스에이운영(주)</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 고양시 덕양구</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>1312660786</t>
+          <t>8738702917</t>
         </is>
       </c>
       <c r="D19" s="2" t="n">
@@ -928,7 +928,7 @@
         <v>0.0</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>70.0</v>
+        <v>12.0</v>
       </c>
       <c r="H19" s="2" t="n">
         <v>0.0</v>
@@ -948,17 +948,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>대한약품공업(주)반월공장</t>
+          <t>영상폴리텍</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>1348500111</t>
+          <t>1312660786</t>
         </is>
       </c>
       <c r="D20" s="2" t="n">
@@ -971,7 +971,7 @@
         <v>0.0</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>82.0</v>
+        <v>70.0</v>
       </c>
       <c r="H20" s="2" t="n">
         <v>0.0</v>
@@ -991,30 +991,30 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>주식회사 대솔오시스</t>
+          <t>대한약품공업(주)반월공장</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>1398115533</t>
+          <t>1348500111</t>
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
       <c r="F21" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G21" s="2" t="n">
-        <v>37.0</v>
+        <v>82.0</v>
       </c>
       <c r="H21" s="2" t="n">
         <v>0.0</v>
@@ -1034,7 +1034,7 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>(주) 대한솔루션</t>
+          <t>주식회사 대솔오시스</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>1398100699</t>
+          <t>1398115533</t>
         </is>
       </c>
       <c r="D22" s="2" t="n">
@@ -1057,7 +1057,7 @@
         <v>0.0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>47.0</v>
+        <v>37.0</v>
       </c>
       <c r="H22" s="2" t="n">
         <v>0.0</v>
@@ -1077,7 +1077,7 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>(주)오성기전</t>
+          <t>(주) 대한솔루션</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>1318629038</t>
+          <t>1398100699</t>
         </is>
       </c>
       <c r="D23" s="2" t="n">
@@ -1100,7 +1100,7 @@
         <v>0.0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>44.0</v>
+        <v>47.0</v>
       </c>
       <c r="H23" s="2" t="n">
         <v>0.0</v>
@@ -1120,30 +1120,30 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>(주)윤성에프앤씨</t>
+          <t>(주)오성기전</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>경기도 안성시</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>1348150350</t>
+          <t>1318629038</t>
         </is>
       </c>
       <c r="D24" s="2" t="n">
-        <v>288.0</v>
+        <v>80.0</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>288.0</v>
+        <v>80.0</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>1.0</v>
+        <v>47.0</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>214.0</v>
+        <v>44.0</v>
       </c>
       <c r="H24" s="2" t="n">
         <v>0.0</v>
@@ -1152,7 +1152,7 @@
         <v>0.0</v>
       </c>
       <c r="J24" s="2" t="n">
-        <v>73.0</v>
+        <v>0.0</v>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
@@ -1163,30 +1163,30 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>(주)백콤</t>
+          <t>(주)윤성에프앤씨</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 남동구</t>
+          <t>경기도 안성시</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>1308628716</t>
+          <t>1348150350</t>
         </is>
       </c>
       <c r="D25" s="2" t="n">
-        <v>47.0</v>
+        <v>288.0</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>47.0</v>
+        <v>288.0</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>10.0</v>
+        <v>1.0</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>27.0</v>
+        <v>217.0</v>
       </c>
       <c r="H25" s="2" t="n">
         <v>0.0</v>
@@ -1195,7 +1195,7 @@
         <v>0.0</v>
       </c>
       <c r="J25" s="2" t="n">
-        <v>0.0</v>
+        <v>73.0</v>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
@@ -1206,39 +1206,39 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>한국미쓰비시엘리베이터(주)</t>
+          <t>(주)백콤</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 연수구</t>
+          <t>인천광역시 남동구</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>1378514007</t>
+          <t>1308628716</t>
         </is>
       </c>
       <c r="D26" s="2" t="n">
-        <v>209.0</v>
+        <v>47.0</v>
       </c>
       <c r="E26" s="2" t="n">
-        <v>209.0</v>
+        <v>47.0</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>92.0</v>
+        <v>10.0</v>
       </c>
       <c r="G26" s="2" t="n">
-        <v>128.0</v>
+        <v>27.0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>10.0</v>
+        <v>0.0</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>17.0</v>
+        <v>0.0</v>
       </c>
       <c r="J26" s="2" t="n">
-        <v>4.0</v>
+        <v>0.0</v>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
@@ -1249,39 +1249,39 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>비카코리아 주식회사</t>
+          <t>한국미쓰비시엘리베이터(주)</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>경기도 오산시</t>
+          <t>인천광역시 연수구</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>6108128707</t>
+          <t>1378514007</t>
         </is>
       </c>
       <c r="D27" s="2" t="n">
-        <v>0.0</v>
+        <v>209.0</v>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0</v>
+        <v>209.0</v>
       </c>
       <c r="F27" s="2" t="n">
-        <v>0.0</v>
+        <v>92.0</v>
       </c>
       <c r="G27" s="2" t="n">
-        <v>107.0</v>
+        <v>123.0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>0.0</v>
+        <v>11.0</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>0.0</v>
+        <v>17.0</v>
       </c>
       <c r="J27" s="2" t="n">
-        <v>0.0</v>
+        <v>6.0</v>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
@@ -1292,39 +1292,39 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>(주)디바이스</t>
+          <t>비카코리아 주식회사</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>충청남도 천안시 서북구</t>
+          <t>경기도 오산시</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>3128157991</t>
+          <t>6108128707</t>
         </is>
       </c>
       <c r="D28" s="2" t="n">
-        <v>70.0</v>
+        <v>157.0</v>
       </c>
       <c r="E28" s="2" t="n">
-        <v>70.0</v>
+        <v>157.0</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>70.0</v>
+        <v>107.0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>17.0</v>
+        <v>2.0</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>0.0</v>
+        <v>7.0</v>
       </c>
       <c r="J28" s="2" t="n">
-        <v>51.0</v>
+        <v>64.0</v>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
@@ -1335,39 +1335,39 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>(주)지에프에스</t>
+          <t>(주)디바이스</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>경기도 의정부시</t>
+          <t>충청남도 천안시 서북구</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>1278107419</t>
+          <t>3128157991</t>
         </is>
       </c>
       <c r="D29" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.0</v>
+        <v>70.0</v>
       </c>
       <c r="F29" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G29" s="2" t="n">
-        <v>104.0</v>
+        <v>70.0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>0.0</v>
+        <v>17.0</v>
       </c>
       <c r="I29" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J29" s="2" t="n">
-        <v>0.0</v>
+        <v>50.0</v>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
@@ -1378,39 +1378,39 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>(주)케이피씨엠</t>
+          <t>(주)지에프에스</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>경상북도 경산시</t>
+          <t>경기도 의정부시</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>5158140973</t>
+          <t>1278107419</t>
         </is>
       </c>
       <c r="D30" s="2" t="n">
-        <v>188.0</v>
+        <v>0.0</v>
       </c>
       <c r="E30" s="2" t="n">
-        <v>188.0</v>
+        <v>0.0</v>
       </c>
       <c r="F30" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>174.0</v>
+        <v>103.0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>25.0</v>
+        <v>0.0</v>
       </c>
       <c r="J30" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
@@ -1421,36 +1421,36 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>(주)경인기술</t>
+          <t>(주)케이피씨엠</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 영등포구</t>
+          <t>경상북도 경산시</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>1138156416</t>
+          <t>5158140973</t>
         </is>
       </c>
       <c r="D31" s="2" t="n">
-        <v>0.0</v>
+        <v>188.0</v>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.0</v>
+        <v>188.0</v>
       </c>
       <c r="F31" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G31" s="2" t="n">
-        <v>35.0</v>
+        <v>174.0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>0.0</v>
+        <v>8.0</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>0.0</v>
+        <v>24.0</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.0</v>
@@ -1464,17 +1464,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>(주)코리아하이텍</t>
+          <t>(주)경인기술</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>경기도 안산시 단원구</t>
+          <t>서울특별시 영등포구</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>1348106311</t>
+          <t>1138156416</t>
         </is>
       </c>
       <c r="D32" s="2" t="n">
@@ -1487,7 +1487,7 @@
         <v>0.0</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>296.0</v>
+        <v>35.0</v>
       </c>
       <c r="H32" s="2" t="n">
         <v>0.0</v>
@@ -1507,30 +1507,30 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>에브제트아시아(주)</t>
+          <t>(주)코리아하이텍</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 강서구</t>
+          <t>경기도 안산시 단원구</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>1208731282</t>
+          <t>1348106311</t>
         </is>
       </c>
       <c r="D33" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="E33" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>70.0</v>
+        <v>286.0</v>
       </c>
       <c r="H33" s="2" t="n">
         <v>0.0</v>
@@ -1550,39 +1550,39 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>디엔엠항공</t>
+          <t>에브제트아시아(주)</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>서울특별시 강서구</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>6131783159</t>
+          <t>1208731282</t>
         </is>
       </c>
       <c r="D34" s="2" t="n">
-        <v>452.0</v>
+        <v>1.0</v>
       </c>
       <c r="E34" s="2" t="n">
-        <v>315.0</v>
+        <v>1.0</v>
       </c>
       <c r="F34" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>243.0</v>
+        <v>70.0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>22.0</v>
+        <v>0.0</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>44.0</v>
+        <v>0.0</v>
       </c>
       <c r="J34" s="2" t="n">
-        <v>3.0</v>
+        <v>0.0</v>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
@@ -1593,39 +1593,39 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>씨트론(주)</t>
+          <t>디엔엠항공</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>인천광역시 계양구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>1228159023</t>
+          <t>6131783159</t>
         </is>
       </c>
       <c r="D35" s="2" t="n">
-        <v>0.0</v>
+        <v>452.0</v>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.0</v>
+        <v>315.0</v>
       </c>
       <c r="F35" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>41.0</v>
+        <v>243.0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>0.0</v>
+        <v>18.0</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>0.0</v>
+        <v>48.0</v>
       </c>
       <c r="J35" s="2" t="n">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
@@ -1636,17 +1636,17 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>(주)알피바이오</t>
+          <t>씨트론(주)</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>경기도 화성시 만세구</t>
+          <t>인천광역시 계양구</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>7758501361</t>
+          <t>1228159023</t>
         </is>
       </c>
       <c r="D36" s="2" t="n">
@@ -1659,7 +1659,7 @@
         <v>0.0</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>10.0</v>
+        <v>41.0</v>
       </c>
       <c r="H36" s="2" t="n">
         <v>0.0</v>
@@ -1679,30 +1679,30 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>주식회사 코젠바이오텍</t>
+          <t>(주)알피바이오</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>서울특별시 금천구</t>
+          <t>경기도 화성시 만세구</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>1018156320</t>
+          <t>7758501361</t>
         </is>
       </c>
       <c r="D37" s="2" t="n">
-        <v>45.0</v>
+        <v>163.0</v>
       </c>
       <c r="E37" s="2" t="n">
-        <v>45.0</v>
+        <v>163.0</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>0.0</v>
+        <v>16.0</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>150.0</v>
+        <v>10.0</v>
       </c>
       <c r="H37" s="2" t="n">
         <v>0.0</v>
@@ -1722,39 +1722,39 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>(주)에어로피스</t>
+          <t>주식회사 코젠바이오텍</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>경기도 김포시</t>
+          <t>서울특별시 금천구</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>1378604165</t>
+          <t>1018156320</t>
         </is>
       </c>
       <c r="D38" s="2" t="n">
-        <v>237.0</v>
+        <v>45.0</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>237.0</v>
+        <v>45.0</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>57.0</v>
+        <v>0.0</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>176.0</v>
+        <v>150.0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>30.0</v>
+        <v>0.0</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>27.0</v>
+        <v>0.0</v>
       </c>
       <c r="J38" s="2" t="n">
-        <v>86.0</v>
+        <v>0.0</v>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
@@ -1765,39 +1765,39 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>주식회사 덱스레보</t>
+          <t>(주)에어로피스</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>서울 금천구</t>
+          <t>경기도 김포시</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>1198678150</t>
+          <t>1378604165</t>
         </is>
       </c>
       <c r="D39" s="2" t="n">
-        <v>10.0</v>
+        <v>237.0</v>
       </c>
       <c r="E39" s="2" t="n">
-        <v>10.0</v>
+        <v>237.0</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>0.0</v>
+        <v>57.0</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>160.0</v>
+        <v>183.0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>0.0</v>
+        <v>30.0</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>0.0</v>
+        <v>27.0</v>
       </c>
       <c r="J39" s="2" t="n">
-        <v>0.0</v>
+        <v>86.0</v>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
@@ -1808,36 +1808,36 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>주식회사 카프마이크로</t>
+          <t>주식회사 덱스레보</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>경남 사천시</t>
+          <t>서울 금천구</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>3148613655</t>
+          <t>1198678150</t>
         </is>
       </c>
       <c r="D40" s="2" t="n">
-        <v>60.0</v>
+        <v>10.0</v>
       </c>
       <c r="E40" s="2" t="n">
-        <v>60.0</v>
+        <v>10.0</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>17.0</v>
+        <v>0.0</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>33.0</v>
+        <v>160.0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>14.0</v>
+        <v>0.0</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.0</v>
@@ -1851,39 +1851,39 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>연합정밀(주)</t>
+          <t>주식회사 카프마이크로</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>충남 천안시 동남구</t>
+          <t>경남 사천시</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>3128109219</t>
+          <t>3148613655</t>
         </is>
       </c>
       <c r="D41" s="2" t="n">
-        <v>1827.0</v>
+        <v>60.0</v>
       </c>
       <c r="E41" s="2" t="n">
-        <v>1827.0</v>
+        <v>60.0</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>525.0</v>
+        <v>17.0</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>7.0</v>
+        <v>23.0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>1.0</v>
+        <v>4.0</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
       <c r="J41" s="2" t="n">
-        <v>18.0</v>
+        <v>2.0</v>
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
@@ -1894,39 +1894,39 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>(주)우리기술</t>
+          <t>연합정밀(주)</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>서울 마포구</t>
+          <t>충남 천안시 동남구</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>1128138619</t>
+          <t>3128109219</t>
         </is>
       </c>
       <c r="D42" s="2" t="n">
-        <v>84.0</v>
+        <v>1827.0</v>
       </c>
       <c r="E42" s="2" t="n">
-        <v>84.0</v>
+        <v>1827.0</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>22.0</v>
+        <v>525.0</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>71.0</v>
+        <v>936.0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
       <c r="I42" s="2" t="n">
         <v>0.0</v>
       </c>
       <c r="J42" s="2" t="n">
-        <v>0.0</v>
+        <v>18.0</v>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
@@ -1937,33 +1937,33 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>(주)신화프리텍</t>
+          <t>(주)우리기술</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>경남 창원시 성산구</t>
+          <t>서울 마포구</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>6088151660</t>
+          <t>1128138619</t>
         </is>
       </c>
       <c r="D43" s="2" t="n">
-        <v>1070.0</v>
+        <v>84.0</v>
       </c>
       <c r="E43" s="2" t="n">
-        <v>1051.0</v>
+        <v>84.0</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>111.0</v>
+        <v>22.0</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>1523.0</v>
+        <v>70.0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>39.0</v>
+        <v>0.0</v>
       </c>
       <c r="I43" s="2" t="n">
         <v>0.0</v>
@@ -1980,39 +1980,39 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>(주)한국기능공사</t>
+          <t>(주)신화프리텍</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>충북 음성군</t>
+          <t>경남 창원시 성산구</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>1258112293</t>
+          <t>6088151660</t>
         </is>
       </c>
       <c r="D44" s="2" t="n">
-        <v>614.0</v>
+        <v>1183.0</v>
       </c>
       <c r="E44" s="2" t="n">
-        <v>614.0</v>
+        <v>1164.0</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>250.0</v>
+        <v>28.0</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>309.0</v>
+        <v>1523.0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>3.0</v>
+        <v>37.0</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>8.0</v>
+        <v>2.0</v>
       </c>
       <c r="J44" s="2" t="n">
-        <v>376.0</v>
+        <v>0.0</v>
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
@@ -2023,39 +2023,39 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>(주)휴니드테크놀러지스</t>
+          <t>(주)한국기능공사</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>인천 연수구</t>
+          <t>충북 음성군</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>1238106174</t>
+          <t>1258112293</t>
         </is>
       </c>
       <c r="D45" s="2" t="n">
-        <v>916.0</v>
+        <v>614.0</v>
       </c>
       <c r="E45" s="2" t="n">
-        <v>916.0</v>
+        <v>614.0</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>128.0</v>
+        <v>250.0</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>871.0</v>
+        <v>309.0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>40.0</v>
+        <v>2.0</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>42.0</v>
+        <v>9.0</v>
       </c>
       <c r="J45" s="2" t="n">
-        <v>145.0</v>
+        <v>376.0</v>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
@@ -2066,41 +2066,84 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>(주)휴니드테크놀러지스</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>인천 연수구</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>1238106174</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="n">
+        <v>916.0</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>916.0</v>
+      </c>
+      <c r="F46" s="2" t="n">
+        <v>128.0</v>
+      </c>
+      <c r="G46" s="2" t="n">
+        <v>871.0</v>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>41.0</v>
+      </c>
+      <c r="I46" s="2" t="n">
+        <v>42.0</v>
+      </c>
+      <c r="J46" s="2" t="n">
+        <v>145.0</v>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
           <t>(주)서연이화 아산공장</t>
         </is>
       </c>
-      <c r="B46" s="2" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>충남 아산시</t>
         </is>
       </c>
-      <c r="C46" s="2" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>3128564374</t>
         </is>
       </c>
-      <c r="D46" s="2" t="n">
-        <v>84.0</v>
-      </c>
-      <c r="E46" s="2" t="n">
-        <v>84.0</v>
-      </c>
-      <c r="F46" s="2" t="n">
+      <c r="D47" s="2" t="n">
+        <v>85.0</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>85.0</v>
+      </c>
+      <c r="F47" s="2" t="n">
         <v>5.0</v>
       </c>
-      <c r="G46" s="2" t="n">
-        <v>47.0</v>
-      </c>
-      <c r="H46" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="I46" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="J46" s="2" t="n">
-        <v>0.0</v>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="G47" s="2" t="n">
+        <v>85.0</v>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I47" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="J47" s="2" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>

</xml_diff>